<commit_message>
alredy send to heroku
</commit_message>
<xml_diff>
--- a/media/DF_COTATION.xlsx
+++ b/media/DF_COTATION.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Visual_Studio\Project_Development\media\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8F504C0-9D37-49EE-B41B-DB7F78E42DA7}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{010C3088-DC70-45FF-BC12-73CCB58CAFF9}" xr6:coauthVersionLast="46" xr6:coauthVersionMax="46" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="21840" windowHeight="13140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="cota" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="132" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="46">
   <si>
     <t>ID</t>
   </si>
@@ -55,15 +55,12 @@
     <t>Projeto Restauração</t>
   </si>
   <si>
-    <t>CFTV</t>
+    <t>CONTROLE DE ACESSO</t>
   </si>
   <si>
     <t>Memorial Descritivo</t>
   </si>
   <si>
-    <t>Memorial Descritivo do Sistema de CFTV</t>
-  </si>
-  <si>
     <t>MD</t>
   </si>
   <si>
@@ -73,12 +70,6 @@
     <t>.DOC / .PDF</t>
   </si>
   <si>
-    <t>30</t>
-  </si>
-  <si>
-    <t>60</t>
-  </si>
-  <si>
     <t>Critérios de Projeto</t>
   </si>
   <si>
@@ -94,9 +85,6 @@
     <t>Folha de Dados</t>
   </si>
   <si>
-    <t>Folha de Dados  do Sistema de CFTV</t>
-  </si>
-  <si>
     <t>FD</t>
   </si>
   <si>
@@ -121,21 +109,12 @@
     <t>A1</t>
   </si>
   <si>
-    <t>1</t>
-  </si>
-  <si>
-    <t>20</t>
-  </si>
-  <si>
     <t>Planta de Locação</t>
   </si>
   <si>
     <t>DE</t>
   </si>
   <si>
-    <t>8</t>
-  </si>
-  <si>
     <t>Planta de Encaminhamento de Cabos</t>
   </si>
   <si>
@@ -167,9 +146,6 @@
   </si>
   <si>
     <t>LM</t>
-  </si>
-  <si>
-    <t>24</t>
   </si>
   <si>
     <t>Requisição de Materiais</t>
@@ -549,9 +525,8 @@
   <cols>
     <col min="1" max="2" width="3" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="34.42578125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="37.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="34.42578125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="15.42578125" bestFit="1" customWidth="1"/>
@@ -597,7 +572,7 @@
         <v>0</v>
       </c>
       <c r="B3">
-        <v>17</v>
+        <v>65</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
@@ -609,22 +584,22 @@
         <v>12</v>
       </c>
       <c r="F3" t="s">
+        <v>12</v>
+      </c>
+      <c r="G3" t="s">
         <v>13</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H3" t="s">
         <v>14</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>15</v>
       </c>
-      <c r="I3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J3" t="s">
-        <v>17</v>
-      </c>
-      <c r="K3" t="s">
-        <v>18</v>
+      <c r="J3">
+        <v>30</v>
+      </c>
+      <c r="K3">
+        <v>50</v>
       </c>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
@@ -632,7 +607,7 @@
         <v>1</v>
       </c>
       <c r="B4">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
         <v>10</v>
@@ -641,25 +616,25 @@
         <v>11</v>
       </c>
       <c r="E4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="F4" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="G4" t="s">
-        <v>20</v>
+        <v>17</v>
       </c>
       <c r="H4" t="s">
+        <v>14</v>
+      </c>
+      <c r="I4" t="s">
         <v>15</v>
       </c>
-      <c r="I4" t="s">
-        <v>16</v>
-      </c>
-      <c r="J4" t="s">
-        <v>17</v>
-      </c>
-      <c r="K4" t="s">
-        <v>18</v>
+      <c r="J4">
+        <v>30</v>
+      </c>
+      <c r="K4">
+        <v>50</v>
       </c>
     </row>
     <row r="5" spans="1:11" x14ac:dyDescent="0.25">
@@ -667,34 +642,34 @@
         <v>2</v>
       </c>
       <c r="B5">
+        <v>67</v>
+      </c>
+      <c r="C5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" t="s">
         <v>19</v>
       </c>
-      <c r="C5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E5" t="s">
-        <v>21</v>
-      </c>
-      <c r="F5" t="s">
-        <v>21</v>
-      </c>
-      <c r="G5" t="s">
-        <v>22</v>
-      </c>
       <c r="H5" t="s">
+        <v>14</v>
+      </c>
+      <c r="I5" t="s">
         <v>15</v>
-      </c>
-      <c r="I5" t="s">
-        <v>16</v>
       </c>
       <c r="J5">
         <v>30</v>
       </c>
       <c r="K5">
-        <v>60</v>
+        <v>50</v>
       </c>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.25">
@@ -702,34 +677,34 @@
         <v>3</v>
       </c>
       <c r="B6">
+        <v>68</v>
+      </c>
+      <c r="C6" t="s">
+        <v>10</v>
+      </c>
+      <c r="D6" t="s">
+        <v>11</v>
+      </c>
+      <c r="E6" t="s">
         <v>20</v>
       </c>
-      <c r="C6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" t="s">
-        <v>11</v>
-      </c>
-      <c r="E6" t="s">
-        <v>23</v>
-      </c>
       <c r="F6" t="s">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="G6" t="s">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="H6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I6" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="J6">
         <v>5</v>
       </c>
       <c r="K6">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="7" spans="1:11" x14ac:dyDescent="0.25">
@@ -737,7 +712,7 @@
         <v>4</v>
       </c>
       <c r="B7">
-        <v>21</v>
+        <v>69</v>
       </c>
       <c r="C7" t="s">
         <v>10</v>
@@ -746,19 +721,19 @@
         <v>11</v>
       </c>
       <c r="E7" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="F7" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="G7" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="H7" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="I7" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -772,7 +747,7 @@
         <v>5</v>
       </c>
       <c r="B8">
-        <v>22</v>
+        <v>70</v>
       </c>
       <c r="C8" t="s">
         <v>10</v>
@@ -781,25 +756,25 @@
         <v>11</v>
       </c>
       <c r="E8" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="F8" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="G8" t="s">
+        <v>24</v>
+      </c>
+      <c r="H8" t="s">
         <v>28</v>
       </c>
-      <c r="H8" t="s">
-        <v>32</v>
-      </c>
       <c r="I8" t="s">
-        <v>30</v>
-      </c>
-      <c r="J8" t="s">
-        <v>33</v>
-      </c>
-      <c r="K8" t="s">
-        <v>34</v>
+        <v>26</v>
+      </c>
+      <c r="J8">
+        <v>1</v>
+      </c>
+      <c r="K8">
+        <v>10</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">
@@ -807,7 +782,7 @@
         <v>6</v>
       </c>
       <c r="B9">
-        <v>23</v>
+        <v>71</v>
       </c>
       <c r="C9" t="s">
         <v>10</v>
@@ -816,25 +791,25 @@
         <v>11</v>
       </c>
       <c r="E9" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="F9" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="G9" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H9" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="I9" t="s">
-        <v>30</v>
-      </c>
-      <c r="J9" t="s">
-        <v>33</v>
-      </c>
-      <c r="K9" t="s">
-        <v>37</v>
+        <v>26</v>
+      </c>
+      <c r="J9">
+        <v>1</v>
+      </c>
+      <c r="K9">
+        <v>10</v>
       </c>
     </row>
     <row r="10" spans="1:11" x14ac:dyDescent="0.25">
@@ -842,7 +817,7 @@
         <v>7</v>
       </c>
       <c r="B10">
-        <v>24</v>
+        <v>72</v>
       </c>
       <c r="C10" t="s">
         <v>10</v>
@@ -851,19 +826,19 @@
         <v>11</v>
       </c>
       <c r="E10" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="F10" t="s">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="G10" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H10" t="s">
-        <v>32</v>
+        <v>28</v>
       </c>
       <c r="I10" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J10">
         <v>1</v>
@@ -877,7 +852,7 @@
         <v>8</v>
       </c>
       <c r="B11">
-        <v>25</v>
+        <v>73</v>
       </c>
       <c r="C11" t="s">
         <v>10</v>
@@ -886,25 +861,25 @@
         <v>11</v>
       </c>
       <c r="E11" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="F11" t="s">
-        <v>39</v>
+        <v>32</v>
       </c>
       <c r="G11" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H11" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="I11" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J11">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="K11">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:11" x14ac:dyDescent="0.25">
@@ -912,34 +887,34 @@
         <v>9</v>
       </c>
       <c r="B12">
+        <v>74</v>
+      </c>
+      <c r="C12" t="s">
+        <v>10</v>
+      </c>
+      <c r="D12" t="s">
+        <v>11</v>
+      </c>
+      <c r="E12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F12" t="s">
+        <v>34</v>
+      </c>
+      <c r="G12" t="s">
+        <v>30</v>
+      </c>
+      <c r="H12" t="s">
+        <v>33</v>
+      </c>
+      <c r="I12" t="s">
         <v>26</v>
       </c>
-      <c r="C12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" t="s">
-        <v>11</v>
-      </c>
-      <c r="E12" t="s">
-        <v>41</v>
-      </c>
-      <c r="F12" t="s">
-        <v>41</v>
-      </c>
-      <c r="G12" t="s">
-        <v>36</v>
-      </c>
-      <c r="H12" t="s">
-        <v>40</v>
-      </c>
-      <c r="I12" t="s">
-        <v>30</v>
-      </c>
       <c r="J12">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="K12">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.25">
@@ -947,7 +922,7 @@
         <v>10</v>
       </c>
       <c r="B13">
-        <v>27</v>
+        <v>75</v>
       </c>
       <c r="C13" t="s">
         <v>10</v>
@@ -956,25 +931,25 @@
         <v>11</v>
       </c>
       <c r="E13" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="F13" t="s">
-        <v>42</v>
+        <v>35</v>
       </c>
       <c r="G13" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="H13" t="s">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="I13" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="J13">
-        <v>6</v>
+        <v>20</v>
       </c>
       <c r="K13">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.25">
@@ -982,7 +957,7 @@
         <v>11</v>
       </c>
       <c r="B14">
-        <v>28</v>
+        <v>76</v>
       </c>
       <c r="C14" t="s">
         <v>10</v>
@@ -991,25 +966,25 @@
         <v>11</v>
       </c>
       <c r="E14" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="F14" t="s">
-        <v>43</v>
+        <v>36</v>
       </c>
       <c r="G14" t="s">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="H14" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I14" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="J14">
         <v>6</v>
       </c>
       <c r="K14">
-        <v>10</v>
+        <v>5</v>
       </c>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.25">
@@ -1017,7 +992,7 @@
         <v>12</v>
       </c>
       <c r="B15">
-        <v>29</v>
+        <v>77</v>
       </c>
       <c r="C15" t="s">
         <v>10</v>
@@ -1026,22 +1001,22 @@
         <v>11</v>
       </c>
       <c r="E15" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="F15" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="G15" t="s">
-        <v>46</v>
+        <v>39</v>
       </c>
       <c r="H15" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I15" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="J15">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="K15">
         <v>10</v>
@@ -1052,34 +1027,34 @@
         <v>13</v>
       </c>
       <c r="B16">
+        <v>78</v>
+      </c>
+      <c r="C16" t="s">
+        <v>10</v>
+      </c>
+      <c r="D16" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" t="s">
+        <v>40</v>
+      </c>
+      <c r="F16" t="s">
+        <v>40</v>
+      </c>
+      <c r="G16" t="s">
+        <v>41</v>
+      </c>
+      <c r="H16" t="s">
+        <v>14</v>
+      </c>
+      <c r="I16" t="s">
+        <v>22</v>
+      </c>
+      <c r="J16">
+        <v>10</v>
+      </c>
+      <c r="K16">
         <v>30</v>
-      </c>
-      <c r="C16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" t="s">
-        <v>11</v>
-      </c>
-      <c r="E16" t="s">
-        <v>47</v>
-      </c>
-      <c r="F16" t="s">
-        <v>47</v>
-      </c>
-      <c r="G16" t="s">
-        <v>48</v>
-      </c>
-      <c r="H16" t="s">
-        <v>15</v>
-      </c>
-      <c r="I16" t="s">
-        <v>26</v>
-      </c>
-      <c r="J16" t="s">
-        <v>37</v>
-      </c>
-      <c r="K16" t="s">
-        <v>49</v>
       </c>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.25">
@@ -1087,7 +1062,7 @@
         <v>14</v>
       </c>
       <c r="B17">
-        <v>31</v>
+        <v>79</v>
       </c>
       <c r="C17" t="s">
         <v>10</v>
@@ -1096,25 +1071,25 @@
         <v>11</v>
       </c>
       <c r="E17" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="F17" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="G17" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="H17" t="s">
+        <v>14</v>
+      </c>
+      <c r="I17" t="s">
         <v>15</v>
       </c>
-      <c r="I17" t="s">
-        <v>16</v>
-      </c>
       <c r="J17">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="K17">
-        <v>10</v>
+        <v>15</v>
       </c>
     </row>
     <row r="18" spans="1:11" x14ac:dyDescent="0.25">
@@ -1122,7 +1097,7 @@
         <v>15</v>
       </c>
       <c r="B18">
-        <v>32</v>
+        <v>80</v>
       </c>
       <c r="C18" t="s">
         <v>10</v>
@@ -1131,25 +1106,25 @@
         <v>11</v>
       </c>
       <c r="E18" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="F18" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
       <c r="G18" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="H18" t="s">
+        <v>14</v>
+      </c>
+      <c r="I18" t="s">
+        <v>22</v>
+      </c>
+      <c r="J18">
         <v>15</v>
       </c>
-      <c r="I18" t="s">
-        <v>26</v>
-      </c>
-      <c r="J18">
-        <v>12</v>
-      </c>
       <c r="K18">
-        <v>10</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>